<commit_message>
Update to version 1.1.7 with bug fixes.
</commit_message>
<xml_diff>
--- a/tests/branch_structures_human.xlsx
+++ b/tests/branch_structures_human.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95CFB6E1-A317-4450-B632-D95099A0135C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F47B04-0325-44CC-A68A-BD4B20A2DB51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
   <si>
     <t>E2F2fF5fe</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -214,6 +214,10 @@
   </si>
   <si>
     <t>0.05*N</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E1e</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -539,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1332E35-274F-4402-9398-6428F590D294}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
@@ -769,6 +773,14 @@
         <v>29</v>
       </c>
     </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>